<commit_message>
Close out Mohonk expense report with parking and confirmed rental car charge
Added OMA short-term parking (Brian Brazeal reimbursement) and confirmed the
final Budget rental car receipt matches the estimate exactly ($468.21, no
variance). Report total now $2,463.56, fully confirmed with no open items.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/travel/trips/2026-08-02_2026-08-09_mohonk-expense-report.xlsx
+++ b/travel/trips/2026-08-02_2026-08-09_mohonk-expense-report.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\peter\Documents\Group-2\travel\trips\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{52D6A045-36A4-48A5-B4A6-25310027A614}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{1856E48E-89F4-4B19-AC94-2DE686EE1BDC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="1749" windowWidth="10577" windowHeight="5365" xr2:uid="{5966F086-6AE1-4065-A4FD-346F3896E491}"/>
+    <workbookView xWindow="2263" yWindow="2263" windowWidth="15428" windowHeight="9454" xr2:uid="{A9DA3FAF-6937-458A-B34B-8010AEEEC99D}"/>
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="2" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="178" uniqueCount="103">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="184" uniqueCount="105">
   <si>
     <t>UNIFOCUS EXPENSE REPORT  |  Mohonk Mountain House</t>
   </si>
@@ -115,7 +115,7 @@
     <t>AA OMA-ORD-EWR (AA GFLPYC), ticket 0012349569454 - cash balance after flight credits, Visa -2674</t>
   </si>
   <si>
-    <t>Budget rental car, VW Atlas Cross Sport AWD, EWR pickup 8/2 2:45PM - return 8/7 5:00PM, agreement U266355924 (est. - confirm final charge/card at drop-off receipt)</t>
+    <t>Budget rental car, VW Atlas Cross Sport AWD, agreement 266355924, EWR pickup 8/2 2:45PM - actual return 8/7 3:37PM, 218 mi driven (odometer 3890-4108), Visa -2674, Net Charges confirmed USD 468.21, Total Due 0.00 - final receipt matches estimate exactly, no variance</t>
   </si>
   <si>
     <t>Car Rental</t>
@@ -178,6 +178,12 @@
     <t>McDonald's #26777 (ORD Terminal 3) - breakfast, layover on return home, Visa -2674</t>
   </si>
   <si>
+    <t>Omaha Eppley Airfield (OMA) short-term parking, entry 8/2 05:41 - exit 8/3 07:46, receipt 13366 - paid by Brian Brazeal (Capital One Visa -9323) who borrowed Pete's car from OMA for the week; Pete to reimburse Brian, claimed on ER</t>
+  </si>
+  <si>
+    <t>Parking</t>
+  </si>
+  <si>
     <t>TOTAL</t>
   </si>
   <si>
@@ -235,7 +241,7 @@
     <t>-2674</t>
   </si>
   <si>
-    <t>Visa SW Rapid Rewards+ (flight cash balance, return flight, Taco Bell, gas, hotel + fees, both Ubers, Scarpetta, Chick Chick, E-ZPass, ORD breakfast)</t>
+    <t>Visa SW Rapid Rewards+ (flight cash balance, return flight, Taco Bell, gas, hotel + fees, both Ubers, Scarpetta, Chick Chick, E-ZPass, ORD breakfast, Budget rental car)</t>
   </si>
   <si>
     <t>SW Credit</t>
@@ -256,10 +262,10 @@
     <t>Visa WF Active Cash (Tallow - Shaver Hall dinner, full billable value; net card charge was .77 after credit)</t>
   </si>
   <si>
-    <t>TBD</t>
-  </si>
-  <si>
-    <t>Budget rental car - confirm card used at drop-off</t>
+    <t>-9323</t>
+  </si>
+  <si>
+    <t>Capital One Visa (Brian Brazeal) - OMA short-term parking, Pete to reimburse Brian</t>
   </si>
   <si>
     <t>OPEN ITEMS BEFORE SUBMISSION</t>
@@ -520,10 +526,10 @@
     <xf numFmtId="49" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="0" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="3" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -883,11 +889,11 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9C638474-0CB8-463C-A475-97FADC8D2292}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F4E1230F-6C72-4073-ACBA-406F7FF36C7C}">
   <sheetPr>
     <tabColor rgb="FF64381F"/>
   </sheetPr>
-  <dimension ref="A1:E34"/>
+  <dimension ref="A1:E35"/>
   <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="22.69140625" customWidth="1"/>
@@ -898,7 +904,7 @@
   <sheetData>
     <row r="1" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A1" s="27" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="B1" s="3"/>
       <c r="C1" s="3"/>
@@ -907,7 +913,7 @@
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A2" s="4" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="B2" s="28" t="s">
         <v>4</v>
@@ -918,10 +924,10 @@
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A3" s="4" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="B3" s="28" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="C3" s="28"/>
       <c r="D3" s="28"/>
@@ -929,10 +935,10 @@
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A4" s="4" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="B4" s="28" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="C4" s="28"/>
       <c r="D4" s="28"/>
@@ -940,7 +946,7 @@
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A5" s="4" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="B5" s="28" t="s">
         <v>18</v>
@@ -951,10 +957,10 @@
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A6" s="4" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="B6" s="28" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="C6" s="28"/>
       <c r="D6" s="28"/>
@@ -962,10 +968,10 @@
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A7" s="4" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="B7" s="28" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="C7" s="28"/>
       <c r="D7" s="28"/>
@@ -973,7 +979,7 @@
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A9" s="29" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="B9" s="3"/>
       <c r="C9" s="3"/>
@@ -988,7 +994,7 @@
         <v>7</v>
       </c>
       <c r="C10" s="30" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.4">
@@ -1081,54 +1087,54 @@
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A19" s="12" t="s">
+        <v>46</v>
+      </c>
+      <c r="B19" s="10">
+        <v>34.5</v>
+      </c>
+      <c r="C19" s="9">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A20" s="31" t="s">
         <v>40</v>
       </c>
-      <c r="B19" s="10">
+      <c r="B20" s="32">
         <v>4.96</v>
       </c>
-      <c r="C19" s="9">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A20" s="25" t="s">
-        <v>59</v>
-      </c>
-      <c r="B20" s="26">
-        <f>SUM(B11:B19)</f>
-        <v>2429.06</v>
-      </c>
-      <c r="C20" s="24"/>
-    </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A22" s="29" t="s">
-        <v>60</v>
-      </c>
-      <c r="B22" s="3"/>
-      <c r="C22" s="3"/>
-      <c r="D22" s="3"/>
-      <c r="E22" s="3"/>
+      <c r="C20" s="33">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A21" s="25" t="s">
+        <v>61</v>
+      </c>
+      <c r="B21" s="26">
+        <f>SUM(B11:B20)</f>
+        <v>2463.56</v>
+      </c>
+      <c r="C21" s="24"/>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A23" s="30" t="s">
-        <v>61</v>
-      </c>
-      <c r="B23" s="30" t="s">
+      <c r="A23" s="29" t="s">
         <v>62</v>
       </c>
-      <c r="C23" s="30" t="s">
+      <c r="B23" s="3"/>
+      <c r="C23" s="3"/>
+      <c r="D23" s="3"/>
+      <c r="E23" s="3"/>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A24" s="30" t="s">
+        <v>63</v>
+      </c>
+      <c r="B24" s="30" t="s">
+        <v>64</v>
+      </c>
+      <c r="C24" s="30" t="s">
         <v>7</v>
-      </c>
-    </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A24" s="34" t="s">
-        <v>63</v>
-      </c>
-      <c r="B24" s="31" t="s">
-        <v>64</v>
-      </c>
-      <c r="C24" s="32">
-        <v>1595.58</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.4">
@@ -1139,7 +1145,7 @@
         <v>66</v>
       </c>
       <c r="C25" s="10">
-        <v>311.8</v>
+        <v>2063.79</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.4">
@@ -1150,7 +1156,7 @@
         <v>68</v>
       </c>
       <c r="C26" s="32">
-        <v>19.850000000000001</v>
+        <v>311.8</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.4">
@@ -1161,7 +1167,7 @@
         <v>70</v>
       </c>
       <c r="C27" s="10">
-        <v>33.619999999999997</v>
+        <v>19.850000000000001</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.4">
@@ -1172,40 +1178,42 @@
         <v>72</v>
       </c>
       <c r="C28" s="32">
-        <v>468.21</v>
+        <v>33.619999999999997</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A29" s="25" t="s">
-        <v>45</v>
-      </c>
-      <c r="B29" s="24"/>
-      <c r="C29" s="26">
-        <f>SUM(C24:C28)</f>
-        <v>2429.0599999999995</v>
-      </c>
-    </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A31" s="35" t="s">
+      <c r="A29" s="13" t="s">
         <v>73</v>
       </c>
-      <c r="B31" s="3"/>
-      <c r="C31" s="3"/>
-      <c r="D31" s="3"/>
-      <c r="E31" s="3"/>
+      <c r="B29" s="12" t="s">
+        <v>74</v>
+      </c>
+      <c r="C29" s="10">
+        <v>34.5</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A30" s="25" t="s">
+        <v>47</v>
+      </c>
+      <c r="B30" s="24"/>
+      <c r="C30" s="26">
+        <f>SUM(C25:C29)</f>
+        <v>2463.56</v>
+      </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A32" s="1" t="s">
-        <v>74</v>
-      </c>
-      <c r="B32" s="1"/>
-      <c r="C32" s="1"/>
-      <c r="D32" s="1"/>
-      <c r="E32" s="1"/>
+      <c r="A32" s="35" t="s">
+        <v>75</v>
+      </c>
+      <c r="B32" s="3"/>
+      <c r="C32" s="3"/>
+      <c r="D32" s="3"/>
+      <c r="E32" s="3"/>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A33" s="1" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B33" s="1"/>
       <c r="C33" s="1"/>
@@ -1214,22 +1222,31 @@
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A34" s="1" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="B34" s="1"/>
       <c r="C34" s="1"/>
       <c r="D34" s="1"/>
       <c r="E34" s="1"/>
     </row>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A35" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="B35" s="1"/>
+      <c r="C35" s="1"/>
+      <c r="D35" s="1"/>
+      <c r="E35" s="1"/>
+    </row>
   </sheetData>
   <mergeCells count="13">
-    <mergeCell ref="A34:E34"/>
+    <mergeCell ref="A35:E35"/>
     <mergeCell ref="B7:E7"/>
     <mergeCell ref="A9:E9"/>
-    <mergeCell ref="A22:E22"/>
-    <mergeCell ref="A31:E31"/>
+    <mergeCell ref="A23:E23"/>
     <mergeCell ref="A32:E32"/>
     <mergeCell ref="A33:E33"/>
+    <mergeCell ref="A34:E34"/>
     <mergeCell ref="A1:E1"/>
     <mergeCell ref="B2:E2"/>
     <mergeCell ref="B3:E3"/>
@@ -1242,11 +1259,11 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FABE12CC-00D8-4186-B6A2-AA99B57CE0A8}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4EFD3B56-7E85-4195-9970-2C10B5C777BD}">
   <sheetPr>
     <tabColor rgb="FFB6752E"/>
   </sheetPr>
-  <dimension ref="A1:J33"/>
+  <dimension ref="A1:J34"/>
   <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="10.69140625" customWidth="1"/>
@@ -1940,24 +1957,38 @@
       </c>
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.4">
-      <c r="A23" s="8"/>
+      <c r="A23" s="8">
+        <v>46236</v>
+      </c>
       <c r="B23" s="9" t="str">
-        <f>IF(A23="","",TEXT(A23,"ddd"))</f>
-        <v/>
-      </c>
-      <c r="C23" s="20"/>
+        <f>TEXT(A23,"ddd")</f>
+        <v>Sun</v>
+      </c>
+      <c r="C23" s="10">
+        <v>34.5</v>
+      </c>
       <c r="D23" s="11">
         <v>1</v>
       </c>
       <c r="E23" s="10">
         <f>C23*D23</f>
-        <v>0</v>
-      </c>
-      <c r="F23" s="12"/>
-      <c r="G23" s="12"/>
-      <c r="H23" s="12"/>
-      <c r="I23" s="12"/>
-      <c r="J23" s="21"/>
+        <v>34.5</v>
+      </c>
+      <c r="F23" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="G23" s="12" t="s">
+        <v>45</v>
+      </c>
+      <c r="H23" s="9" t="s">
+        <v>46</v>
+      </c>
+      <c r="I23" s="12" t="s">
+        <v>18</v>
+      </c>
+      <c r="J23" s="13" t="s">
+        <v>19</v>
+      </c>
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A24" s="14"/>
@@ -1965,7 +1996,7 @@
         <f>IF(A24="","",TEXT(A24,"ddd"))</f>
         <v/>
       </c>
-      <c r="C24" s="22"/>
+      <c r="C24" s="20"/>
       <c r="D24" s="17">
         <v>1</v>
       </c>
@@ -1977,7 +2008,7 @@
       <c r="G24" s="18"/>
       <c r="H24" s="18"/>
       <c r="I24" s="18"/>
-      <c r="J24" s="23"/>
+      <c r="J24" s="21"/>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A25" s="8"/>
@@ -1985,7 +2016,7 @@
         <f>IF(A25="","",TEXT(A25,"ddd"))</f>
         <v/>
       </c>
-      <c r="C25" s="20"/>
+      <c r="C25" s="22"/>
       <c r="D25" s="11">
         <v>1</v>
       </c>
@@ -1997,7 +2028,7 @@
       <c r="G25" s="12"/>
       <c r="H25" s="12"/>
       <c r="I25" s="12"/>
-      <c r="J25" s="21"/>
+      <c r="J25" s="23"/>
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A26" s="14"/>
@@ -2005,7 +2036,7 @@
         <f>IF(A26="","",TEXT(A26,"ddd"))</f>
         <v/>
       </c>
-      <c r="C26" s="22"/>
+      <c r="C26" s="20"/>
       <c r="D26" s="17">
         <v>1</v>
       </c>
@@ -2017,7 +2048,7 @@
       <c r="G26" s="18"/>
       <c r="H26" s="18"/>
       <c r="I26" s="18"/>
-      <c r="J26" s="23"/>
+      <c r="J26" s="21"/>
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A27" s="8"/>
@@ -2025,7 +2056,7 @@
         <f>IF(A27="","",TEXT(A27,"ddd"))</f>
         <v/>
       </c>
-      <c r="C27" s="20"/>
+      <c r="C27" s="22"/>
       <c r="D27" s="11">
         <v>1</v>
       </c>
@@ -2037,7 +2068,7 @@
       <c r="G27" s="12"/>
       <c r="H27" s="12"/>
       <c r="I27" s="12"/>
-      <c r="J27" s="21"/>
+      <c r="J27" s="23"/>
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A28" s="14"/>
@@ -2045,7 +2076,7 @@
         <f>IF(A28="","",TEXT(A28,"ddd"))</f>
         <v/>
       </c>
-      <c r="C28" s="22"/>
+      <c r="C28" s="20"/>
       <c r="D28" s="17">
         <v>1</v>
       </c>
@@ -2057,7 +2088,7 @@
       <c r="G28" s="18"/>
       <c r="H28" s="18"/>
       <c r="I28" s="18"/>
-      <c r="J28" s="23"/>
+      <c r="J28" s="21"/>
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A29" s="8"/>
@@ -2065,7 +2096,7 @@
         <f>IF(A29="","",TEXT(A29,"ddd"))</f>
         <v/>
       </c>
-      <c r="C29" s="20"/>
+      <c r="C29" s="22"/>
       <c r="D29" s="11">
         <v>1</v>
       </c>
@@ -2077,7 +2108,7 @@
       <c r="G29" s="12"/>
       <c r="H29" s="12"/>
       <c r="I29" s="12"/>
-      <c r="J29" s="21"/>
+      <c r="J29" s="23"/>
     </row>
     <row r="30" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A30" s="14"/>
@@ -2085,7 +2116,7 @@
         <f>IF(A30="","",TEXT(A30,"ddd"))</f>
         <v/>
       </c>
-      <c r="C30" s="22"/>
+      <c r="C30" s="20"/>
       <c r="D30" s="17">
         <v>1</v>
       </c>
@@ -2097,7 +2128,7 @@
       <c r="G30" s="18"/>
       <c r="H30" s="18"/>
       <c r="I30" s="18"/>
-      <c r="J30" s="23"/>
+      <c r="J30" s="21"/>
     </row>
     <row r="31" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A31" s="8"/>
@@ -2105,7 +2136,7 @@
         <f>IF(A31="","",TEXT(A31,"ddd"))</f>
         <v/>
       </c>
-      <c r="C31" s="20"/>
+      <c r="C31" s="22"/>
       <c r="D31" s="11">
         <v>1</v>
       </c>
@@ -2117,7 +2148,7 @@
       <c r="G31" s="12"/>
       <c r="H31" s="12"/>
       <c r="I31" s="12"/>
-      <c r="J31" s="21"/>
+      <c r="J31" s="23"/>
     </row>
     <row r="32" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A32" s="14"/>
@@ -2125,7 +2156,7 @@
         <f>IF(A32="","",TEXT(A32,"ddd"))</f>
         <v/>
       </c>
-      <c r="C32" s="22"/>
+      <c r="C32" s="20"/>
       <c r="D32" s="17">
         <v>1</v>
       </c>
@@ -2137,34 +2168,54 @@
       <c r="G32" s="18"/>
       <c r="H32" s="18"/>
       <c r="I32" s="18"/>
-      <c r="J32" s="23"/>
+      <c r="J32" s="21"/>
     </row>
     <row r="33" spans="1:10" x14ac:dyDescent="0.4">
-      <c r="A33" s="24"/>
-      <c r="B33" s="24"/>
-      <c r="C33" s="24"/>
-      <c r="D33" s="25" t="s">
-        <v>45</v>
-      </c>
-      <c r="E33" s="26">
-        <f>SUM(E5:E32)</f>
-        <v>2429.06</v>
-      </c>
-      <c r="F33" s="24"/>
-      <c r="G33" s="24"/>
-      <c r="H33" s="24"/>
-      <c r="I33" s="24"/>
-      <c r="J33" s="24"/>
+      <c r="A33" s="8"/>
+      <c r="B33" s="9" t="str">
+        <f>IF(A33="","",TEXT(A33,"ddd"))</f>
+        <v/>
+      </c>
+      <c r="C33" s="22"/>
+      <c r="D33" s="11">
+        <v>1</v>
+      </c>
+      <c r="E33" s="10">
+        <f>C33*D33</f>
+        <v>0</v>
+      </c>
+      <c r="F33" s="12"/>
+      <c r="G33" s="12"/>
+      <c r="H33" s="12"/>
+      <c r="I33" s="12"/>
+      <c r="J33" s="23"/>
+    </row>
+    <row r="34" spans="1:10" x14ac:dyDescent="0.4">
+      <c r="A34" s="24"/>
+      <c r="B34" s="24"/>
+      <c r="C34" s="24"/>
+      <c r="D34" s="25" t="s">
+        <v>47</v>
+      </c>
+      <c r="E34" s="26">
+        <f>SUM(E5:E33)</f>
+        <v>2463.56</v>
+      </c>
+      <c r="F34" s="24"/>
+      <c r="G34" s="24"/>
+      <c r="H34" s="24"/>
+      <c r="I34" s="24"/>
+      <c r="J34" s="24"/>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:J1"/>
   </mergeCells>
   <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F5:F32" xr:uid="{C6ECC75D-C667-48BE-8075-0549477EADB0}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F5:F33" xr:uid="{E6D9AE04-0F43-46AA-863D-F00E64B85D66}">
       <formula1>"UF,PERSONAL,OTHER"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H5:H32" xr:uid="{356F0088-ABF6-48BD-8B50-E14A627CFCF8}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H5:H33" xr:uid="{B0661D6E-323E-45D4-981F-EA9E6E27243F}">
       <formula1>"Air Fare,Taxi/Train/Bus,Car Rental,Gas/Tolls,Parking,Hotel,Bkfst,Lunch,Dinner,Phone/Data,Computer,Other,Postage,Misc"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2173,7 +2224,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DD867586-0F30-4DEB-BB51-E9E5E6E9A6AE}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2318F84D-DF98-4C5B-B25F-41AB49DE6C53}">
   <sheetPr>
     <tabColor rgb="FFF0E4D6"/>
   </sheetPr>
@@ -2185,132 +2236,132 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A1" s="4" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A7" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A8" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A9" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A11" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A12" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A13" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A14" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A15" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A16" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A17" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A18" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A19" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A20" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A22" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A23" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A24" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
     </row>
     <row r="26" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A26" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
     </row>
     <row r="27" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A27" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
     </row>
     <row r="28" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A28" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
     </row>
     <row r="29" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A29" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
     </row>
     <row r="30" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A30" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Reconcile Mohonk ER against source receipts and build the first receipt packet
- Corrected ER: caught a missing $17.04 Uber tip (return ride actually
  totaled $130.69, charged as 2 separate transactions), confirmed hotel
  fees against the actual property folio, combined the Uber charge back
  onto one line. Total now $2,480.60, every line source-documented.
- Archived all 20 processed receipts into the OneDrive year-folder
  (not tracked in git per the established workflow)
- Built the working Python/pypdf/Pillow receipt-packet pipeline after
  confirming Acrobat COM automation is a dead end on this machine's
  64-bit Acrobat; corrected page-margin math to respect the letterhead's
  header/footer safe zone
- First successful packet build: 39 pages, Unifocus Contractor\Mohonk folder

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/travel/trips/2026-08-02_2026-08-09_mohonk-expense-report.xlsx
+++ b/travel/trips/2026-08-02_2026-08-09_mohonk-expense-report.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\peter\Documents\Group-2\travel\trips\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{5F51C584-A73E-42D0-8761-0D9095DCD0B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{7EC3ABDD-310A-45DE-B94B-6C00EDDCFD16}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2263" yWindow="2263" windowWidth="15428" windowHeight="9454" xr2:uid="{6A06982B-AC92-48BF-8175-DAEB804979ED}"/>
+    <workbookView xWindow="2263" yWindow="2263" windowWidth="15428" windowHeight="9454" xr2:uid="{130B8C68-8788-4F3A-B927-7780531E84BE}"/>
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="2" r:id="rId1"/>
@@ -193,10 +193,10 @@
     <t>Other</t>
   </si>
   <si>
-    <t>Uber, Hotel Seville Nomad (3:01 AM) to EWR Terminal A (3:33 AM), UberX, driver Muhammad, 19.45 mi/31 min</t>
-  </si>
-  <si>
-    <t>Hotel Seville Nomad - mandatory fees, folio checkout ~4:17 AM (after physical departure via Uber) (Destination Fee /night x2 + NYC taxes), Hyatt folio 2529375976</t>
+    <t>Uber, Hotel Seville Nomad (3:01 AM) to EWR Terminal A (3:33 AM), UberX, driver Muhammad, 19.45 mi/31 min - fare+fees .65 + tip .04 (charged as 2 separate transactions 1 minute apart, combined here on one line)</t>
+  </si>
+  <si>
+    <t>Hotel Seville Nomad - mandatory fees, confirmed via property folio (Destination Fee /night x2 + NYC Sales Tax 8.875% + NYC Occupancy Tax 5.875%), Hyatt folio/confirmation 2529375976</t>
   </si>
   <si>
     <t>McDonald's #26777 (ORD Terminal 3, 6:56 AM) - breakfast, layover on return home</t>
@@ -271,7 +271,7 @@
     <t>-2674</t>
   </si>
   <si>
-    <t>Visa SW Rapid Rewards+ (flight cash balance, return flight, Taco Bell, gas, hotel + fees, both Ubers, Scarpetta, Chick Chick, E-ZPass, ORD breakfast, Budget rental car)</t>
+    <t>Visa SW Rapid Rewards+ (flight cash balance, return flight, Taco Bell, gas, hotel + fees, both Ubers + separate return tip, Scarpetta, Chick Chick, E-ZPass, ORD breakfast, Budget rental car)</t>
   </si>
   <si>
     <t>SW Credit</t>
@@ -922,7 +922,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{304F2538-6469-4F3D-933C-8B1D9CACBFBB}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E75F4965-0C6F-47B7-8C7E-053EB55B29C1}">
   <sheetPr>
     <tabColor rgb="FF64381F"/>
   </sheetPr>
@@ -1090,7 +1090,7 @@
         <v>41</v>
       </c>
       <c r="B16" s="33">
-        <v>242.79</v>
+        <v>259.83</v>
       </c>
       <c r="C16" s="34">
         <v>2</v>
@@ -1168,7 +1168,7 @@
       </c>
       <c r="B23" s="27">
         <f>SUM(B13:B22)</f>
-        <v>2463.56</v>
+        <v>2480.6</v>
       </c>
       <c r="C23" s="25"/>
     </row>
@@ -1200,7 +1200,7 @@
         <v>76</v>
       </c>
       <c r="C27" s="11">
-        <v>2063.79</v>
+        <v>2080.83</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.4">
@@ -1254,7 +1254,7 @@
       <c r="B32" s="25"/>
       <c r="C32" s="27">
         <f>SUM(C27:C31)</f>
-        <v>2463.56</v>
+        <v>2480.6</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.4">
@@ -1316,7 +1316,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0AA6B548-1C31-4F3A-87A5-7F6E227AC84F}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{70D64207-5B4D-42B3-9328-76414D9B2897}">
   <sheetPr>
     <tabColor rgb="FFB6752E"/>
   </sheetPr>
@@ -2026,14 +2026,14 @@
         <v>Sun</v>
       </c>
       <c r="C21" s="11">
-        <v>113.65</v>
+        <v>130.69</v>
       </c>
       <c r="D21" s="12">
         <v>1</v>
       </c>
       <c r="E21" s="11">
         <f>C21*D21</f>
-        <v>113.65</v>
+        <v>130.69</v>
       </c>
       <c r="F21" s="10" t="s">
         <v>16</v>
@@ -2360,7 +2360,7 @@
       </c>
       <c r="E34" s="27">
         <f>SUM(E5:E33)</f>
-        <v>2463.5600000000004</v>
+        <v>2480.6000000000004</v>
       </c>
       <c r="F34" s="25"/>
       <c r="G34" s="25"/>
@@ -2375,10 +2375,10 @@
     <mergeCell ref="A1:L1"/>
   </mergeCells>
   <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F5:F33" xr:uid="{17B99C76-54A6-48D6-B9FB-132AC1406B11}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F5:F33" xr:uid="{C2D18644-9A7C-49B6-988A-EF8C6E1D1EF6}">
       <formula1>"UF,PERSONAL,OTHER"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H5:H33" xr:uid="{BBED7A34-6F31-4F29-A43B-5EE0B31170A0}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H5:H33" xr:uid="{4B445555-14E1-4BAD-9E77-5BDEC98C5494}">
       <formula1>"Air Fare,Taxi/Train/Bus,Car Rental,Gas/Tolls,Parking,Hotel,Bkfst,Lunch,Dinner,Phone/Data,Computer,Other,Postage,Misc"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2387,7 +2387,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{56389F32-CAE4-4001-8F12-3B12E6DC2BD4}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FF7B1A7B-A31B-458D-9579-F0014AB1728D}">
   <sheetPr>
     <tabColor rgb="FFF0E4D6"/>
   </sheetPr>

</xml_diff>